<commit_message>
adding lab 2 and 3
</commit_message>
<xml_diff>
--- a/project/Lab_02_rubric.xlsx
+++ b/project/Lab_02_rubric.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -678,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.1640625" customWidth="1"/>
@@ -705,160 +705,194 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="34" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="15">
+    <row r="2" spans="1:8" ht="33.75" customHeight="1" thickBot="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>1.1 Import Your Saved Data from Lab 1</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>import() from the rio package used to import the data file exported at the end of Lab 1</t>
+        </is>
+      </c>
+      <c r="C2" s="4">
         <v>0.5</v>
       </c>
       <c r="D2" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="15">
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Sections</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>1.1 Import Your Saved Data from Lab 1</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Result saved as a new object called wbns_00</t>
+        </is>
+      </c>
+      <c r="C3" s="4">
         <v>0.5</v>
       </c>
       <c r="D3" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>31</v>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>1.1 Import Your Saved Data from Lab 1</t>
+        </is>
       </c>
       <c r="G3" s="9">
         <f>SUM(IF($D$2=FALSE(),0,1)*$C$2,IF($D$3=FALSE(),0,1)*$C$3,IF($D$4=FALSE(),0,1)*$C$4)</f>
-        <v>0</v>
       </c>
       <c r="H3" s="10">
         <f>SUM($C$2:$C$4)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="15">
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>1.1 Import Your Saved Data from Lab 1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>dim() (or similar) used to print the number of rows and columns to verify the import</t>
+        </is>
+      </c>
+      <c r="C4" s="4">
         <v>1</v>
       </c>
       <c r="D4" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>35</v>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>1.2 Filtering to Target Subpopulation</t>
+        </is>
       </c>
       <c r="G4" s="9">
         <f>SUM(IF($D$5=FALSE(),0,1)*$C$5,IF($D$6=FALSE(),0,1)*$C$6,IF($D$7=FALSE(),0,1)*$C$7)</f>
-        <v>0</v>
       </c>
       <c r="H4" s="10">
         <f>SUM($C$5:$C$7)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="17">
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="50" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>1.2 Filtering to Target Subpopulation</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Pipeline uses filter() (and filter_out() for Project 2) with logical conditions that correctly match the student's chosen project's population (Project 1 includes received free groceries/meals)</t>
+        </is>
+      </c>
+      <c r="C5" s="11">
         <v>1.5</v>
       </c>
       <c r="D5" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>36</v>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>1.3 Selecting Project Variables</t>
+        </is>
       </c>
       <c r="G5" s="9">
         <f>SUM(IF($D$8=FALSE(),0,1)*$C$8,IF($D$9=FALSE(),0,1)*$C$9,IF($D$10=FALSE(),0,1)*$C$10)</f>
-        <v>0</v>
       </c>
       <c r="H5" s="10">
         <f>SUM($C$8:$C$10)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="17">
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>1.2 Filtering to Target Subpopulation</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Result saved as a new object called wbns_01_pop</t>
+        </is>
+      </c>
+      <c r="C6" s="11">
         <v>0.5</v>
       </c>
       <c r="D6" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>37</v>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>1.4 Rename Variables for Clarity</t>
+        </is>
       </c>
       <c r="G6" s="9">
-        <f>SUM(IF($D$11=FALSE(),0,1)*$C$11,IF($D$12=FALSE(),0,1)*$C$12)</f>
-        <v>0</v>
+        <f>SUM(IF($D$11=FALSE(),0,1)*$C$11,IF($D$12=FALSE(),0,1)*$C$12,IF($D$13=FALSE(),0,1)*$C$13)</f>
       </c>
       <c r="H6" s="10">
-        <f>SUM($C$11:$C$12)</f>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="17">
+        <f>SUM($C$11:$C$13)</f>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>1.2 Filtering to Target Subpopulation</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Number of rows printed before and after filtering to verify the operation</t>
+        </is>
+      </c>
+      <c r="C7" s="11">
         <v>1</v>
       </c>
       <c r="D7" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>38</v>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
       </c>
       <c r="G7" s="9">
-        <f>SUM(IF($D$13=FALSE(),0,1)*$C$13,IF($D$14=FALSE(),0,1)*$C$14,IF($D$15=FALSE(),0,1)*$C$15)</f>
-        <v>0</v>
+        <f>SUM(IF($D$14=FALSE(),0,1)*$C$14,IF($D$15=FALSE(),0,1)*$C$15,IF($D$16=FALSE(),0,1)*$C$16,IF($D$17=FALSE(),0,1)*$C$17,IF($D$18=FALSE(),0,1)*$C$18,IF($D$19=FALSE(),0,1)*$C$19)</f>
       </c>
       <c r="H7" s="10">
-        <f>SUM($C$13:$C$15)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>10</v>
+        <f>SUM($C$14:$C$19)</f>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="50" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>1.3 Selecting Project Variables</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>select() used to reduce the data frame to ID variables, population variables, main variables, and additional variables (or 0-3 reasonable substitutes/additions)</t>
+        </is>
       </c>
       <c r="C8" s="4">
         <v>1.5</v>
@@ -866,24 +900,28 @@
       <c r="D8" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>39</v>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>1.6 Handle Missing Data</t>
+        </is>
       </c>
       <c r="G8" s="9">
-        <f>SUM(IF($D$16=FALSE(),0,1)*$C$16,IF($D$17=FALSE(),0,1)*$C$17,IF($D$18=FALSE(),0,1)*$C$18)</f>
-        <v>0</v>
+        <f>SUM(IF($D$20=FALSE(),0,1)*$C$20,IF($D$21=FALSE(),0,1)*$C$21,IF($D$22=FALSE(),0,1)*$C$22,IF($D$23=FALSE(),0,1)*$C$23)</f>
       </c>
       <c r="H8" s="10">
-        <f>SUM($C$16:$C$18)</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>11</v>
+        <f>SUM($C$20:$C$23)</f>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1.3 Selecting Project Variables</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Result saved as a new object called wbns_02_pop_vars</t>
+        </is>
       </c>
       <c r="C9" s="4">
         <v>0.5</v>
@@ -891,24 +929,28 @@
       <c r="D9" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>40</v>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>1.7 Export Datasets</t>
+        </is>
       </c>
       <c r="G9" s="9">
-        <f>SUM(IF($D$19=FALSE(),0,1)*$C$19,IF($D$20=FALSE(),0,1)*$C$20,IF($D$21=FALSE(),0,1)*$C$21,IF($D$22=FALSE(),0,1)*$C$22)</f>
-        <v>0</v>
+        <f>SUM(IF($D$24=FALSE(),0,1)*$C$24,IF($D$25=FALSE(),0,1)*$C$25,IF($D$26=FALSE(),0,1)*$C$26)</f>
       </c>
       <c r="H9" s="10">
-        <f>SUM($C$19:$C$22)</f>
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>12</v>
+        <f>SUM($C$24:$C$26)</f>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1.3 Selecting Project Variables</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Number of columns printed before and after selecting to verify the operation</t>
+        </is>
       </c>
       <c r="C10" s="4">
         <v>1</v>
@@ -916,214 +958,266 @@
       <c r="D10" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>41</v>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>1.8 AI Use Statement</t>
+        </is>
       </c>
       <c r="G10" s="9">
-        <f>SUM(IF($D$23=FALSE(),0,1)*$C$23,IF($D$24=FALSE(),0,1)*$C$24,IF($D$25=FALSE(),0,1)*$C$25)</f>
-        <v>0</v>
+        <f>SUM(IF($D$27=FALSE(),0,1)*$C$27)</f>
       </c>
       <c r="H10" s="10">
-        <f>SUM($C$23:$C$25)</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="17">
-        <v>1</v>
+        <f>SUM($C$27:$C$27)</f>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>1.4 Rename Variables for Clarity</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>rename() used with the required names for main variables (per the project's tab) and clear, snake_case names for additional variables</t>
+        </is>
+      </c>
+      <c r="C11" s="11">
+        <v>1.5</v>
       </c>
       <c r="D11" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>15</v>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>General / Document Quality</t>
+        </is>
       </c>
       <c r="G11" s="9">
-        <f>SUM(IF($D$26=FALSE(),0,1)*$C$26,IF($D$27=FALSE(),0,1)*$C$27,IF($D$28=FALSE(),0,1)*$C$28,IF($D$29=FALSE(),0,1)*$C$29)</f>
-        <v>0</v>
+        <f>SUM(IF($D$28=FALSE(),0,1)*$C$28,IF($D$29=FALSE(),0,1)*$C$29,IF($D$30=FALSE(),0,1)*$C$30,IF($D$31=FALSE(),0,1)*$C$31)</f>
       </c>
       <c r="H11" s="10">
-        <f>SUM($C$26:$C$29)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="17">
-        <v>1.5</v>
+        <f>SUM($C$28:$C$31)</f>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="33.75" customHeight="1" thickBot="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>1.4 Rename Variables for Clarity</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Result saved as a new object called wbns_03_renamed</t>
+        </is>
+      </c>
+      <c r="C12" s="11">
+        <v>0.5</v>
       </c>
       <c r="D12" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>17</v>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
       </c>
       <c r="G12" s="13">
         <f>SUM(G3:G11)</f>
-        <v>0</v>
       </c>
       <c r="H12" s="14">
         <f>SUM(H3:H11)</f>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="4">
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>1.4 Rename Variables for Clarity</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>glimpse() used afterward to confirm new variable names, with output visible</t>
+        </is>
+      </c>
+      <c r="C13" s="11">
+        <v>1</v>
+      </c>
+      <c r="D13" s="18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>n_miss() and prop_miss() used to report overall missingness</t>
+        </is>
+      </c>
+      <c r="C14" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D14" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>miss_var_summary() (piped into gt()) used to show missingness by variable</t>
+        </is>
+      </c>
+      <c r="C15" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>vis_miss() and gg_miss_upset() plots created</t>
+        </is>
+      </c>
+      <c r="C16" s="4">
+        <v>1</v>
+      </c>
+      <c r="D16" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Project-specific step completed (Projects 2 and 3: gg_miss_fct() plot(s) with the correct fct variable)</t>
+        </is>
+      </c>
+      <c r="C17" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>tabyl() used on each main variable to find hidden missing values (Refused / Don't know)</t>
+        </is>
+      </c>
+      <c r="C18" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="50" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>1.5 Explore Missing Data</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>4-6 sentence paragraph summarizing which variables are most missing, what's missing together, likely reasons (refusals vs. skip logic), and which values need to become NA</t>
+        </is>
+      </c>
+      <c r="C19" s="4">
         <v>1.5</v>
       </c>
-      <c r="D13" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D14" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" s="4">
+      <c r="D19" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>1.6 Handle Missing Data</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Part A: replace_with_na() used to turn Refused / Don't know responses into NA; result saved as wbns_04_na_recoded</t>
+        </is>
+      </c>
+      <c r="C20" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="D20" s="18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>1.6 Handle Missing Data</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Part A: Recoding checked with tabyl() and miss_var_summary()</t>
+        </is>
+      </c>
+      <c r="C21" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D21" s="18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="50" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>1.6 Handle Missing Data</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Part B: drop_na() used on only the project's key variables (Project 3 does NOT drop on skip-logic variables or WIC); result saved as wbns_04_no_na</t>
+        </is>
+      </c>
+      <c r="C22" s="11">
         <v>1</v>
       </c>
-      <c r="D15" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D16" s="18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="11">
-        <v>1</v>
-      </c>
-      <c r="D17" s="18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="11">
-        <v>1</v>
-      </c>
-      <c r="D18" s="18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="4">
-        <v>2</v>
-      </c>
-      <c r="D19" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="D20" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D21" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="4">
-        <v>1.5</v>
-      </c>
-      <c r="D22" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>42</v>
+      <c r="D22" s="18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>1.6 Handle Missing Data</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Part B: Row counts printed before/after, with 1-2 sentences describing how many rows were lost and whether that's reasonable</t>
+        </is>
       </c>
       <c r="C23" s="11">
         <v>1</v>
@@ -1132,68 +1226,88 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="11">
+    <row r="24" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>1.7 Export Datasets</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>export() from the rio package used to save datasets in a .rda file</t>
+        </is>
+      </c>
+      <c r="C24" s="4">
+        <v>1</v>
+      </c>
+      <c r="D24" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>1.7 Export Datasets</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>All four required datasets included: wbns_01_pop, wbns_02_pop_vars, wbns_03_renamed, wbns_04_no_na</t>
+        </is>
+      </c>
+      <c r="C25" s="4">
         <v>1.5</v>
       </c>
-      <c r="D24" s="18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="11">
+      <c r="D25" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>1.7 Export Datasets</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>File saved in the data_project/data_processed folder with a clear, identifiable file name</t>
+        </is>
+      </c>
+      <c r="C26" s="4">
         <v>1</v>
       </c>
-      <c r="D25" s="18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26" s="4">
-        <v>0.5</v>
-      </c>
       <c r="D26" s="16" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D27" s="16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>29</v>
+    <row r="27" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>1.8 AI Use Statement</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>AI Use Statement included (either describing AI use or stating AI was not used)</t>
+        </is>
+      </c>
+      <c r="C27" s="11">
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Editing file is the correct, unmodified .qmd template -- no instructional text/sections deleted</t>
+        </is>
       </c>
       <c r="C28" s="4">
         <v>0.5</v>
@@ -1202,17 +1316,57 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>30</v>
+    <row r="29" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>File renders (knits) without errors</t>
+        </is>
       </c>
       <c r="C29" s="4">
         <v>0.5</v>
       </c>
       <c r="D29" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>File follows naming convention: lastname_firstinit_lab_02.qmd</t>
+        </is>
+      </c>
+      <c r="C30" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D30" s="16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="33.75" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Code is reasonably readable/organized (chunks labeled, no leftover scratch code)</t>
+        </is>
+      </c>
+      <c r="C31" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="16" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>